<commit_message>
Add track summary and no-choice reporting
</commit_message>
<xml_diff>
--- a/готовое_решение/выход/результат_распределения.xlsx
+++ b/готовое_решение/выход/результат_распределения.xlsx
@@ -3,6 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="Результат" sheetId="1" r:id="rId1"/>
+    <sheet name="Количество_по_трекам" sheetId="2" r:id="rId2"/>
+    <sheet name="Без_выбора" sheetId="3" r:id="rId3"/>
+    <sheet name="Приоритеты_1_2" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -68,6 +71,21 @@
           <t>рейтинг</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>выбор трека</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>статус без выбора</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>приоритеты</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -86,6 +104,16 @@
       <c r="D2">
         <v>100.004745</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -104,6 +132,21 @@
       <c r="D3">
         <v>100.004709</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -122,6 +165,16 @@
       <c r="D4">
         <v>100.004707</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -140,6 +193,16 @@
       <c r="D5">
         <v>100.004695</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Трек А: 1, Трек В: 3, Трек С: 2</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -158,6 +221,21 @@
       <c r="D6">
         <v>100.004692</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -176,6 +254,16 @@
       <c r="D7">
         <v>100.004678</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -194,6 +282,16 @@
       <c r="D8">
         <v>100.004652</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -212,6 +310,16 @@
       <c r="D9">
         <v>99.492396</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -230,6 +338,21 @@
       <c r="D10">
         <v>99.492375</v>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -248,6 +371,16 @@
       <c r="D11">
         <v>98.980001</v>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Трек А: 2, Трек В: 1, Трек С: 3</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -266,6 +399,16 @@
       <c r="D12">
         <v>98.394134</v>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -284,6 +427,16 @@
       <c r="D13">
         <v>98.144175</v>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Трек А: 2, Трек В: 1, Трек С: 3</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -302,6 +455,21 @@
       <c r="D14">
         <v>97.987142</v>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -320,6 +488,16 @@
       <c r="D15">
         <v>97.977431</v>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Трек А: 1, Трек В: 3, Трек С: 2</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -338,6 +516,16 @@
       <c r="D16">
         <v>97.798501</v>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -356,6 +544,16 @@
       <c r="D17">
         <v>96.95281</v>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -374,6 +572,21 @@
       <c r="D18">
         <v>96.805618</v>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -392,6 +605,16 @@
       <c r="D19">
         <v>96.283648</v>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -410,6 +633,16 @@
       <c r="D20">
         <v>96.283595</v>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -428,6 +661,16 @@
       <c r="D21">
         <v>96.18788</v>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Трек А: 1, Трек В: 3, Трек С: 2</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -446,6 +689,16 @@
       <c r="D22">
         <v>96.126582</v>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Трек А: 1, Трек В: 2, Трек С: 3</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -464,6 +717,21 @@
       <c r="D23">
         <v>95.028425</v>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -482,6 +750,16 @@
       <c r="D24">
         <v>94.935252</v>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Трек А: 2, Трек В: 3, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -500,6 +778,16 @@
       <c r="D25">
         <v>94.829885</v>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Трек А: 2, Трек В: 1, Трек С: 3</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -518,6 +806,16 @@
       <c r="D26">
         <v>92.905499</v>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Трек А: 2, Трек В: 1, Трек С: 3</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -536,6 +834,16 @@
       <c r="D27">
         <v>92.665237</v>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Трек А: 2, Трек В: 3, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -554,6 +862,16 @@
       <c r="D28">
         <v>92.645695</v>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Трек А: 1, Трек В: 2, Трек С: 3</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -572,6 +890,16 @@
       <c r="D29">
         <v>92.415213</v>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Трек А: 2, Трек В: 3, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -590,6 +918,16 @@
       <c r="D30">
         <v>92.41519</v>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -608,6 +946,16 @@
       <c r="D31">
         <v>88.777326</v>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -626,6 +974,16 @@
       <c r="D32">
         <v>88.671995</v>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -644,6 +1002,16 @@
       <c r="D33">
         <v>87.669419</v>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Трек А: 1, Трек В: 2, Трек С: 3</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -662,6 +1030,16 @@
       <c r="D34">
         <v>87.166744</v>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Трек А: 2, Трек В: 1, Трек С: 3</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -680,6 +1058,21 @@
       <c r="D35">
         <v>87.061286</v>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -698,6 +1091,16 @@
       <c r="D36">
         <v>84.134543</v>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Трек А: 1, Трек В: 2, Трек С: 3</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -716,6 +1119,16 @@
       <c r="D37">
         <v>83.945751</v>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -734,6 +1147,21 @@
       <c r="D38">
         <v>83.014029</v>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -752,6 +1180,16 @@
       <c r="D39">
         <v>80.580077</v>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Трек А: 1, Трек В: 3, Трек С: 2</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -770,6 +1208,21 @@
       <c r="D40">
         <v>79.032891</v>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -788,6 +1241,16 @@
       <c r="D41">
         <v>78.488894</v>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Трек А: 2, Трек В: 3, Трек С: 1</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -806,6 +1269,21 @@
       <c r="D42">
         <v>77.704375</v>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -823,6 +1301,426 @@
       </c>
       <c r="D43">
         <v>77.223957</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>трек</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>назначено студентов</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>приоритет 1 или 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>8</v>
+      </c>
+      <c r="D2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Трек В</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>14</v>
+      </c>
+      <c r="C3">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Трек С</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id ученика</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>трек</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>место в рейтинге</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>рейтинг</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>статус без выбора</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>637756</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>100.004709</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>366609</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Трек В</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>100.004692</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>449867</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>9</v>
+      </c>
+      <c r="D4">
+        <v>99.492375</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>302756</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>13</v>
+      </c>
+      <c r="D5">
+        <v>97.987142</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>254592</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>17</v>
+      </c>
+      <c r="D6">
+        <v>96.805618</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>473699</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Трек С</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>22</v>
+      </c>
+      <c r="D7">
+        <v>95.028425</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>406855</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C8">
+        <v>34</v>
+      </c>
+      <c r="D8">
+        <v>87.061286</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>754466</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Трек В</t>
+        </is>
+      </c>
+      <c r="C9">
+        <v>37</v>
+      </c>
+      <c r="D9">
+        <v>83.014029</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>921709</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Трек В</t>
+        </is>
+      </c>
+      <c r="C10">
+        <v>39</v>
+      </c>
+      <c r="D10">
+        <v>79.032891</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>190122</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C11">
+        <v>41</v>
+      </c>
+      <c r="D11">
+        <v>77.704375</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>трек</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>количество студентов с приоритетом 1 или 2</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>id студентов с приоритетом 1 или 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>17</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>494162, 714473, 497747, 303636, 232693, 530117, 226735, 527662, 381726, 843668, 581151, 702975, 564334, 331430, 898624, 951986, 375035</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Трек В</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>24</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>979609, 596500, 604388, 313703, 874990, 714473, 592028, 497747, 956875, 746559, 968944, 586604, 530117, 527662, 381726, 581151, 363222, 249335, 894613, 564334, 331430, 898624, 523389, 121139</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Трек С</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>23</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>979609, 596500, 494162, 604388, 313703, 874990, 592028, 303636, 956875, 746559, 968944, 586604, 232693, 226735, 843668, 702975, 363222, 249335, 894613, 523389, 951986, 375035, 121139</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>